<commit_message>
Accueil : paires de spécialités BTS ↔ HND (CDC 3.10, maquette)
- Specialite.equivalent : lien symétrique vers la spécialité de l'autre examen,
  posé par apparier() (une seule équivalente, ancien lien défait), contrôlé à
  l'enregistrement ; dans l'administration, le choix se fait d'un côté.
- Migration : CGE↔ACC, BF↔BAF, MCV↔MKT, IG↔SWE si les deux existent ; données
  de démo appariées aussi.
- Classeur du référentiel : colonne facultative « Équivalent (code dans l'autre
  examen) » (un classeur commencé sans elle reste valable), erreurs à la ligne ;
  modèle contenu/referentiel-a-remplir.xlsx régénéré.
- Accueil : chaque carte montre l'équivalente (« HND · Accountancy »), chacune
  vers ses sujets ; en anglais, le HND d'abord.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/contenu/referentiel-a-remplir.xlsx
+++ b/contenu/referentiel-a-remplir.xlsx
@@ -438,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A23"/>
+  <dimension ref="A1:A25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -509,78 +509,92 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Matières — une matière appartient à un seul examen (Comptabilité générale au BTS, Financial Accounting au HND).</t>
+          <t>Équivalent (facultatif) : le code de la spécialité correspondante de l'autre examen (CGE ↔ ACC) ; une seule</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Coefficients — une ligne par couple spécialité / matière ; la matière est écrite comme dans la feuille Matières.</t>
+          <t>des deux lignes suffit.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Chapitres — facultatif ; sert aux quiz par chapitre.</t>
+          <t>Matières — une matière appartient à un seul examen (Comptabilité générale au BTS, Financial Accounting au HND).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Coefficients — une ligne par couple spécialité / matière ; la matière est écrite comme dans la feuille Matières.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Chapitres — facultatif ; sert aux quiz par chapitre.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
           <t>L'import ne supprime jamais rien et peut être relancé avec le même fichier : il met à jour ce qui a changé.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+    <row r="18">
+      <c r="A18" t="inlineStr">
         <is>
           <t>Il vérifie d'abord tout le fichier ; à la moindre erreur, il donne la feuille et la ligne et n'enregistre rien.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Exemples (à recopier dans les feuilles, pas à laisser ici) :</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>Sessions : BTS | 2025 | 14/04/2025 | 27/06/2025</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>Spécialités : BTS | CGE | Comptabilité et gestion des entreprises | Accounting and Business Management | Commerciale | 1</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Matières : BTS | Comptabilité générale | Financial Accounting</t>
+          <t>Sessions : BTS | 2025 | 14/04/2025 | 27/06/2025</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Coefficients : BTS | CGE | Comptabilité générale | 4</t>
+          <t>Spécialités : BTS | CGE | Comptabilité et gestion des entreprises | Accounting and Business Management | Commerciale | 1 | ACC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
+        <is>
+          <t>Matières : BTS | Comptabilité générale | Financial Accounting</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Coefficients : BTS | CGE | Comptabilité générale | 4</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
         <is>
           <t>Chapitres : BTS | Comptabilité générale | 1 | Les amortissements | Depreciation</t>
         </is>
@@ -650,7 +664,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:G1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -659,6 +673,7 @@
     <col width="45" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -690,6 +705,11 @@
       <c r="F1" s="4" t="inlineStr">
         <is>
           <t>Ordre d'affichage</t>
+        </is>
+      </c>
+      <c r="G1" s="4" t="inlineStr">
+        <is>
+          <t>Équivalent (code dans l'autre examen)</t>
         </is>
       </c>
     </row>

</xml_diff>